<commit_message>
Assembly 6B.2 — Intl true-up: Global-e + SG/AU verified, narrative revised
Global-e confirmed inside Shopify dashboard export (no additional GMV).
Amazon SG 2026 = $0; Amazon AU 2026 = A$74.44 (~$48 USD, one sale);
Amazon MX 2026 H1 = MX$907 (~$50 USD). Total intl add: ~$100 (negligible).
2025 SG/AU already captured in locked $513,987 (no change).

2026 H1 GMV: $106,311 → $106,411 (+$100 intl, rounding-level).
Trajectory narrative revised: honest continuing DTC normalization story
(annualized $184–213K vs 2025 $514K); removed "re-accelerating" framing.
Atlantic Access: no change per owner.

Updated: GMV_2026_YTD.md (open items closed), Splitflask_Deal_Memo.md
(narrative revised, table updated), Splitflask_Deal_Workbook.xlsx
(3-Year trend intl cell, Notes & Sources, 2026 Momentum, Summary).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Downloads/Splitflask-Financials/deliverables/Splitflask_Deal_Workbook.xlsx
+++ b/Downloads/Splitflask-Financials/deliverables/Splitflask_Deal_Workbook.xlsx
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>106312</v>
+        <v>106411</v>
       </c>
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n">
@@ -893,7 +893,7 @@
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>PRELIMINARY ⚠</t>
+          <t>PRELIMINARY ⚠ (intl B2 verified)</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>212600</v>
+        <v>212822</v>
       </c>
       <c r="C9" s="17" t="n"/>
       <c r="D9" s="17" t="n"/>
@@ -1623,7 +1623,7 @@
         <v>15940</v>
       </c>
       <c r="D9" s="41" t="n">
-        <v>3000</v>
+        <v>100</v>
       </c>
       <c r="E9" s="39" t="n">
         <v>0</v>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G9" s="32" t="inlineStr">
         <is>
-          <t>2025: Amazon SG/AU $2,383, intl wires $7,686, Best Buy/Walmart $1,111, other. 2026: est.</t>
+          <t>2025: Amazon SG/AU $2,383, intl wires $7,686, Best Buy/Walmart $1,111. 2026 H1: ~$100 actual (SG=$0; AU=$48; MX=$50) — immaterial. Global-e verified inside Shopify export.</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
         <v>513987</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>109311</v>
+        <v>106411</v>
       </c>
       <c r="E10" s="42" t="n">
         <v>1</v>
@@ -1673,7 +1673,7 @@
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="43" t="inlineStr">
         <is>
-          <t>NARRATIVE: 2025 dip = TRANSITION YEAR (entity restructure SGM→SPLT; TikTok wind-down $155K→$25K). NOT a demand decline — Amazon and Shopify cores held. 2026 re-accelerating post-Shark Tank / Kendra deal; wholesale + intl open items likely additive. The $86K wholesale channel in 2024/2025 has no 2026 data yet.</t>
+          <t>NARRATIVE: 2025 dip = TRANSITION YEAR (entity restructure SGM→SPLT; TikTok wind-down $155K→$25K). NOT a demand decline — Amazon and Shopify cores held. 2026 shows continuing DTC channel normalization: core annualized $184–213K vs 2025 $514K. Honest story = softening DTC; wholesale ($84K/yr) + Best Buy/Walmart + Kendra distribution are the 2026+ growth levers not in run-rate. Global-e confirmed inside Shopify (no add). SG/AU 2026 H1 negligible (~$98 total).</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="G9" s="32" t="inlineStr">
         <is>
-          <t>⚠ Global-E intl Shopify pmt $5.4K — may be additive</t>
+          <t>✓ Global-E inside Shopify export (confirmed B2). Not additive.</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1939,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Amazon US + Shopify net + TikTok. Wholesale + Intl + Global-E open (additive).</t>
+          <t>Amazon US + Shopify net + TikTok. ✓ Global-E in Shopify. SG/AU ~$100 (immaterial). Wholesale open.</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="55" t="inlineStr">
         <is>
-          <t>2026 H1 ~$106K — PRELIMINARY</t>
+          <t>2026 H1 ~$106K — PRELIMINARY (OPEN ITEMS CLOSED B2): Platform-sourced (Amazon Sales Dashboard, Shopify export, TikTok PDFs). NOT held to tax-grade footing. Unaudited. CLOSED: (1) Global-E international — CONFIRMED INSIDE Shopify export; bank math consistent (payout split domestic/intl confirms orders already in dashboard). (2) Amazon SG 2026 = $0 sales. Amazon AU 2026 = A$74.44 ($48 USD, one sale Jan 1). Amazon MX 2026 = MX$907 (~$50 USD). Total intl add = ~$100 — negligible. (3) Atlantic Access = NO CHANGE per owner. REMAINING OPEN: Wholesale 2026 status unconfirmed ($84K channel in 2025).</t>
         </is>
       </c>
       <c r="B11" s="56" t="inlineStr">

</xml_diff>